<commit_message>
Add final HTML and PDF reports for capstone submission
</commit_message>
<xml_diff>
--- a/reports/02_Statistical_Analysis_Results.xlsx
+++ b/reports/02_Statistical_Analysis_Results.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,28 +550,28 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C2" t="n">
-        <v>38745.688</v>
+        <v>19511.221</v>
       </c>
       <c r="D2" t="n">
-        <v>228615.347</v>
+        <v>10033.589</v>
       </c>
       <c r="E2" t="n">
         <v>6577</v>
       </c>
       <c r="F2" t="n">
-        <v>12054</v>
+        <v>12019.5</v>
       </c>
       <c r="G2" t="n">
-        <v>16775</v>
+        <v>16749.5</v>
       </c>
       <c r="H2" t="n">
-        <v>23925</v>
+        <v>23854.5</v>
       </c>
       <c r="I2" t="n">
-        <v>2731571</v>
+        <v>65913</v>
       </c>
     </row>
     <row r="3">
@@ -581,25 +581,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C3" t="n">
-        <v>64.54900000000001</v>
+        <v>64.548</v>
       </c>
       <c r="D3" t="n">
-        <v>6.088</v>
+        <v>6.11</v>
       </c>
       <c r="E3" t="n">
         <v>52.2</v>
       </c>
       <c r="F3" t="n">
-        <v>59.9</v>
+        <v>59.875</v>
       </c>
       <c r="G3" t="n">
         <v>63.6</v>
       </c>
       <c r="H3" t="n">
-        <v>69.09999999999999</v>
+        <v>69.125</v>
       </c>
       <c r="I3" t="n">
         <v>86.59999999999999</v>
@@ -612,22 +612,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C4" t="n">
         <v>59.272</v>
       </c>
       <c r="D4" t="n">
-        <v>6.492</v>
+        <v>6.516</v>
       </c>
       <c r="E4" t="n">
         <v>47.3</v>
       </c>
       <c r="F4" t="n">
-        <v>54.7</v>
+        <v>54.675</v>
       </c>
       <c r="G4" t="n">
-        <v>58.6</v>
+        <v>58.55</v>
       </c>
       <c r="H4" t="n">
         <v>64.3</v>
@@ -643,13 +643,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" t="n">
-        <v>8.303000000000001</v>
+        <v>8.304</v>
       </c>
       <c r="D5" t="n">
-        <v>1.89</v>
+        <v>1.897</v>
       </c>
       <c r="E5" t="n">
         <v>4.5</v>
@@ -661,7 +661,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>9.6</v>
+        <v>9.625</v>
       </c>
       <c r="I5" t="n">
         <v>14.6</v>
@@ -670,465 +670,279 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Bachelors_Degree</t>
+          <t>Core_Housing_Need</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C6" t="n">
-        <v>7583.475</v>
+        <v>1720.143</v>
       </c>
       <c r="D6" t="n">
-        <v>44803.637</v>
+        <v>1002.878</v>
       </c>
       <c r="E6" t="n">
-        <v>445</v>
+        <v>115</v>
       </c>
       <c r="F6" t="n">
-        <v>2060</v>
+        <v>967.5</v>
       </c>
       <c r="G6" t="n">
-        <v>3265</v>
+        <v>1432.5</v>
       </c>
       <c r="H6" t="n">
-        <v>4400</v>
+        <v>2287.5</v>
       </c>
       <c r="I6" t="n">
-        <v>534610</v>
+        <v>5335</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>No_Diploma</t>
+          <t>Unaffordable_Housing</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C7" t="n">
-        <v>7958.546</v>
+        <v>35.072</v>
       </c>
       <c r="D7" t="n">
-        <v>46969.835</v>
+        <v>6.939</v>
       </c>
       <c r="E7" t="n">
-        <v>1190</v>
+        <v>17.5</v>
       </c>
       <c r="F7" t="n">
-        <v>2380</v>
+        <v>31.075</v>
       </c>
       <c r="G7" t="n">
-        <v>3385</v>
+        <v>35.6</v>
       </c>
       <c r="H7" t="n">
-        <v>5205</v>
+        <v>38.525</v>
       </c>
       <c r="I7" t="n">
-        <v>561090</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Immigrant_Population</t>
+          <t>Low_Income_AfterTax_Pct</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C8" t="n">
-        <v>17957.518</v>
+        <v>19.514</v>
       </c>
       <c r="D8" t="n">
-        <v>106032.039</v>
+        <v>7.891</v>
       </c>
       <c r="E8" t="n">
-        <v>1795</v>
+        <v>4.5</v>
       </c>
       <c r="F8" t="n">
-        <v>4645</v>
+        <v>14.1</v>
       </c>
       <c r="G8" t="n">
-        <v>7520</v>
+        <v>18.55</v>
       </c>
       <c r="H8" t="n">
-        <v>11425</v>
+        <v>23.95</v>
       </c>
       <c r="I8" t="n">
-        <v>1266005</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Visible_Minority</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9" t="n">
-        <v>19657.589</v>
+        <v>19.209</v>
       </c>
       <c r="D9" t="n">
-        <v>116175.097</v>
+        <v>7.164</v>
       </c>
       <c r="E9" t="n">
-        <v>1100</v>
+        <v>5.28</v>
       </c>
       <c r="F9" t="n">
-        <v>3635</v>
+        <v>13.935</v>
       </c>
       <c r="G9" t="n">
-        <v>7270</v>
+        <v>19.287</v>
       </c>
       <c r="H9" t="n">
-        <v>12700</v>
+        <v>24.384</v>
       </c>
       <c r="I9" t="n">
-        <v>1385855</v>
+        <v>41.388</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Renters</t>
+          <t>No_Diploma_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C10" t="n">
-        <v>7458.369</v>
+        <v>20.331</v>
       </c>
       <c r="D10" t="n">
-        <v>44069.119</v>
+        <v>3.897</v>
       </c>
       <c r="E10" t="n">
-        <v>280</v>
+        <v>11.946</v>
       </c>
       <c r="F10" t="n">
-        <v>1955</v>
+        <v>17.425</v>
       </c>
       <c r="G10" t="n">
-        <v>3235</v>
+        <v>20.979</v>
       </c>
       <c r="H10" t="n">
-        <v>4350</v>
+        <v>23.532</v>
       </c>
       <c r="I10" t="n">
-        <v>525835</v>
+        <v>27.707</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Core_Housing_Need</t>
+          <t>Immigrant_Population_Pct</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C11" t="n">
-        <v>3415.603</v>
+        <v>44.221</v>
       </c>
       <c r="D11" t="n">
-        <v>20157.257</v>
+        <v>13.496</v>
       </c>
       <c r="E11" t="n">
-        <v>115</v>
+        <v>19.59</v>
       </c>
       <c r="F11" t="n">
-        <v>970</v>
+        <v>31.644</v>
       </c>
       <c r="G11" t="n">
-        <v>1435</v>
+        <v>45.355</v>
       </c>
       <c r="H11" t="n">
-        <v>2325</v>
+        <v>55.46</v>
       </c>
       <c r="I11" t="n">
-        <v>240780</v>
+        <v>70.828</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Unaffordable_Housing</t>
+          <t>Visible_Minority_Pct</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C12" t="n">
-        <v>35.083</v>
+        <v>46.48</v>
       </c>
       <c r="D12" t="n">
-        <v>6.916</v>
+        <v>21.963</v>
       </c>
       <c r="E12" t="n">
-        <v>17.5</v>
+        <v>11.865</v>
       </c>
       <c r="F12" t="n">
-        <v>31.1</v>
+        <v>27.239</v>
       </c>
       <c r="G12" t="n">
-        <v>35.7</v>
+        <v>42.516</v>
       </c>
       <c r="H12" t="n">
-        <v>38.5</v>
+        <v>66.08199999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>56.5</v>
+        <v>94.705</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Lone_Parent_Families</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C13" t="n">
-        <v>2164.894</v>
+        <v>18.972</v>
       </c>
       <c r="D13" t="n">
-        <v>12775.943</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>220</v>
+        <v>2.095</v>
       </c>
       <c r="F13" t="n">
-        <v>640</v>
+        <v>13.557</v>
       </c>
       <c r="G13" t="n">
-        <v>870</v>
+        <v>17.655</v>
       </c>
       <c r="H13" t="n">
-        <v>1365</v>
+        <v>23.749</v>
       </c>
       <c r="I13" t="n">
-        <v>152595</v>
+        <v>46.253</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Low_Income_AfterTax_Pct</t>
+          <t>Lone_Parent_Families_Pct</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C14" t="n">
-        <v>19.518</v>
+        <v>5.593</v>
       </c>
       <c r="D14" t="n">
-        <v>7.863</v>
+        <v>1.849</v>
       </c>
       <c r="E14" t="n">
-        <v>4.5</v>
+        <v>2.425</v>
       </c>
       <c r="F14" t="n">
-        <v>14.2</v>
+        <v>4.169</v>
       </c>
       <c r="G14" t="n">
-        <v>18.6</v>
+        <v>5.465</v>
       </c>
       <c r="H14" t="n">
-        <v>23.8</v>
+        <v>6.525</v>
       </c>
       <c r="I14" t="n">
-        <v>45.5</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Bachelors_Degree_Pct</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>141</v>
-      </c>
-      <c r="C15" t="n">
-        <v>19.212</v>
-      </c>
-      <c r="D15" t="n">
-        <v>7.139</v>
-      </c>
-      <c r="E15" t="n">
-        <v>5.28</v>
-      </c>
-      <c r="F15" t="n">
-        <v>13.938</v>
-      </c>
-      <c r="G15" t="n">
-        <v>19.304</v>
-      </c>
-      <c r="H15" t="n">
-        <v>24.379</v>
-      </c>
-      <c r="I15" t="n">
-        <v>41.388</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>No_Diploma_Pct</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>141</v>
-      </c>
-      <c r="C16" t="n">
-        <v>20.333</v>
-      </c>
-      <c r="D16" t="n">
-        <v>3.883</v>
-      </c>
-      <c r="E16" t="n">
-        <v>11.946</v>
-      </c>
-      <c r="F16" t="n">
-        <v>17.431</v>
-      </c>
-      <c r="G16" t="n">
-        <v>20.903</v>
-      </c>
-      <c r="H16" t="n">
-        <v>23.53</v>
-      </c>
-      <c r="I16" t="n">
-        <v>27.707</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Immigrant_Population_Pct</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>141</v>
-      </c>
-      <c r="C17" t="n">
-        <v>44.236</v>
-      </c>
-      <c r="D17" t="n">
-        <v>13.449</v>
-      </c>
-      <c r="E17" t="n">
-        <v>19.59</v>
-      </c>
-      <c r="F17" t="n">
-        <v>31.672</v>
-      </c>
-      <c r="G17" t="n">
-        <v>45.441</v>
-      </c>
-      <c r="H17" t="n">
-        <v>55.444</v>
-      </c>
-      <c r="I17" t="n">
-        <v>70.828</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Visible_Minority_Pct</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>141</v>
-      </c>
-      <c r="C18" t="n">
-        <v>46.51</v>
-      </c>
-      <c r="D18" t="n">
-        <v>21.887</v>
-      </c>
-      <c r="E18" t="n">
-        <v>11.865</v>
-      </c>
-      <c r="F18" t="n">
-        <v>27.263</v>
-      </c>
-      <c r="G18" t="n">
-        <v>42.528</v>
-      </c>
-      <c r="H18" t="n">
-        <v>66.027</v>
-      </c>
-      <c r="I18" t="n">
-        <v>94.705</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Renters_Pct</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>141</v>
-      </c>
-      <c r="C19" t="n">
-        <v>18.973</v>
-      </c>
-      <c r="D19" t="n">
-        <v>8.938000000000001</v>
-      </c>
-      <c r="E19" t="n">
-        <v>2.095</v>
-      </c>
-      <c r="F19" t="n">
-        <v>13.598</v>
-      </c>
-      <c r="G19" t="n">
-        <v>17.67</v>
-      </c>
-      <c r="H19" t="n">
-        <v>23.464</v>
-      </c>
-      <c r="I19" t="n">
-        <v>46.253</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Lone_Parent_Families_Pct</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>141</v>
-      </c>
-      <c r="C20" t="n">
-        <v>5.593</v>
-      </c>
-      <c r="D20" t="n">
-        <v>1.842</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2.425</v>
-      </c>
-      <c r="F20" t="n">
-        <v>4.173</v>
-      </c>
-      <c r="G20" t="n">
-        <v>5.467</v>
-      </c>
-      <c r="H20" t="n">
-        <v>6.499</v>
-      </c>
-      <c r="I20" t="n">
         <v>11.619</v>
       </c>
     </row>
@@ -1143,7 +957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1193,7 +1007,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.734</v>
+        <v>0.735</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -1315,11 +1129,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>No_Diploma_Pct</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.367</v>
+        <v>-0.318</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1333,54 +1147,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.318</v>
+        <v>0.169</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.045</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>p &lt; 0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Core_Housing_Need</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.6830000000000001</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>p = 0.683</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.862</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>p = 0.862</t>
+          <t>p = 0.045</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1427,7 +1205,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.76</v>
+        <v>0.758</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -1445,7 +1223,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.745</v>
+        <v>0.746</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -1463,7 +1241,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -1477,11 +1255,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Core_Housing_Need</t>
+          <t>Immigrant_Population_Pct</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.647</v>
+        <v>0.614</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -1495,11 +1273,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Immigrant_Population_Pct</t>
+          <t>Employment_Rate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.615</v>
+        <v>-0.518</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -1513,11 +1291,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
+          <t>Lone_Parent_Families_Pct</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.52</v>
+        <v>0.503</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -1531,11 +1309,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lone_Parent_Families_Pct</t>
+          <t>Participation_Rate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.503</v>
+        <v>-0.452</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1549,11 +1327,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.452</v>
+        <v>0.403</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -1567,11 +1345,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>No_Diploma_Pct</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.403</v>
+        <v>-0.377</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1585,52 +1363,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Renters_Pct</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.402</v>
+        <v>0.29</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="D11" t="inlineStr">
-        <is>
-          <t>p &lt; 0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Bachelors_Degree_Pct</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>-0.376</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>p &lt; 0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="inlineStr">
         <is>
           <t>p &lt; 0.001</t>
         </is>
@@ -1647,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,12 +1410,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Absolute_Difference</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Consistency</t>
+          <t>Difference</t>
         </is>
       </c>
     </row>
@@ -1687,15 +1424,10 @@
         <v>0.775</v>
       </c>
       <c r="C2" t="n">
-        <v>0.745</v>
+        <v>0.746</v>
       </c>
       <c r="D2" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>0.029</v>
       </c>
     </row>
     <row r="3">
@@ -1705,18 +1437,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.734</v>
+        <v>0.735</v>
       </c>
       <c r="C3" t="n">
-        <v>0.76</v>
+        <v>0.758</v>
       </c>
       <c r="D3" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>-0.023</v>
       </c>
     </row>
     <row r="4">
@@ -1729,15 +1456,10 @@
         <v>0.662</v>
       </c>
       <c r="C4" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="D4" t="n">
-        <v>0.057</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>-0.055</v>
       </c>
     </row>
     <row r="5">
@@ -1750,15 +1472,10 @@
         <v>0.5610000000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>0.615</v>
+        <v>0.614</v>
       </c>
       <c r="D5" t="n">
-        <v>0.054</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>-0.053</v>
       </c>
     </row>
     <row r="6">
@@ -1771,15 +1488,10 @@
         <v>-0.473</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.52</v>
+        <v>-0.518</v>
       </c>
       <c r="D6" t="n">
-        <v>0.047</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>0.045</v>
       </c>
     </row>
     <row r="7">
@@ -1792,15 +1504,10 @@
         <v>0.471</v>
       </c>
       <c r="C7" t="n">
-        <v>0.402</v>
+        <v>0.403</v>
       </c>
       <c r="D7" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>0.068</v>
       </c>
     </row>
     <row r="8">
@@ -1816,12 +1523,7 @@
         <v>0.503</v>
       </c>
       <c r="D8" t="n">
-        <v>0.073</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>-0.073</v>
       </c>
     </row>
     <row r="9">
@@ -1839,94 +1541,37 @@
       <c r="D9" t="n">
         <v>0.06</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>No_Diploma_Pct</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.367</v>
+        <v>-0.318</v>
       </c>
       <c r="C10" t="n">
-        <v>0.403</v>
+        <v>-0.377</v>
       </c>
       <c r="D10" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+        <v>0.059</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.318</v>
+        <v>0.169</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.376</v>
+        <v>0.29</v>
       </c>
       <c r="D11" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Core_Housing_Need</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.647</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.275</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
+        <v>-0.121</v>
       </c>
     </row>
   </sheetData>
@@ -1940,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1967,7 +1612,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3229.724</v>
+        <v>2958.368</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1982,7 +1627,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2443.505</v>
+        <v>2242.616</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1997,7 +1642,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>117.554</v>
+        <v>105.971</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -2008,11 +1653,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Immigrant_Population_Pct</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8.952999999999999</v>
+        <v>7.265</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2027,7 +1672,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.981</v>
+        <v>7.191</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2038,11 +1683,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Immigrant_Population_Pct</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.273</v>
+        <v>5.866</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2057,7 +1702,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.275</v>
+        <v>5.22</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2068,58 +1713,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>No_Diploma_Pct</t>
+          <t>Unaffordable_Housing</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5.222</v>
+        <v>4.428</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Unaffordable_Housing</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4.444</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Renters_Pct</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>4.005</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Core_Housing_Need</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1.021</v>
-      </c>
-      <c r="C12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>

</xml_diff>

<commit_message>
Complete CIND820 capstone project and update documentation
</commit_message>
<xml_diff>
--- a/reports/02_Statistical_Analysis_Results.xlsx
+++ b/reports/02_Statistical_Analysis_Results.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Descriptive_Statistics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Pearson_Correlation" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Spearman_Correlation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparison" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="VIF_Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="VIF_Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Feature_Selection" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Model_Performance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,451 +499,441 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>Participation_Rate</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>std</t>
+          <t>Employment_Rate</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>Unemployment_Rate</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>Core_Housing_Need</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>Unaffordable_Housing</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>Low_Income_AfterTax_Pct</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>Bachelors_Degree_Pct</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>No_Diploma_Pct</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Immigrant_Population_Pct</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Visible_Minority_Pct</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Renters_Pct</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Lone_Parent_Families_Pct</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>count</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>140</v>
       </c>
       <c r="C2" t="n">
-        <v>19511.221</v>
+        <v>140</v>
       </c>
       <c r="D2" t="n">
-        <v>10033.589</v>
+        <v>140</v>
       </c>
       <c r="E2" t="n">
-        <v>6577</v>
+        <v>140</v>
       </c>
       <c r="F2" t="n">
-        <v>12019.5</v>
+        <v>140</v>
       </c>
       <c r="G2" t="n">
-        <v>16749.5</v>
+        <v>140</v>
       </c>
       <c r="H2" t="n">
-        <v>23854.5</v>
+        <v>140</v>
       </c>
       <c r="I2" t="n">
-        <v>65913</v>
+        <v>140</v>
+      </c>
+      <c r="J2" t="n">
+        <v>140</v>
+      </c>
+      <c r="K2" t="n">
+        <v>140</v>
+      </c>
+      <c r="L2" t="n">
+        <v>140</v>
+      </c>
+      <c r="M2" t="n">
+        <v>140</v>
+      </c>
+      <c r="N2" t="n">
+        <v>140</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>140</v>
+        <v>19511.221</v>
       </c>
       <c r="C3" t="n">
         <v>64.548</v>
       </c>
       <c r="D3" t="n">
-        <v>6.11</v>
+        <v>59.272</v>
       </c>
       <c r="E3" t="n">
-        <v>52.2</v>
+        <v>8.304</v>
       </c>
       <c r="F3" t="n">
-        <v>59.875</v>
+        <v>1720.143</v>
       </c>
       <c r="G3" t="n">
-        <v>63.6</v>
+        <v>35.072</v>
       </c>
       <c r="H3" t="n">
-        <v>69.125</v>
+        <v>19.514</v>
       </c>
       <c r="I3" t="n">
-        <v>86.59999999999999</v>
+        <v>19.209</v>
+      </c>
+      <c r="J3" t="n">
+        <v>20.331</v>
+      </c>
+      <c r="K3" t="n">
+        <v>44.221</v>
+      </c>
+      <c r="L3" t="n">
+        <v>46.48</v>
+      </c>
+      <c r="M3" t="n">
+        <v>18.972</v>
+      </c>
+      <c r="N3" t="n">
+        <v>5.593</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
+          <t>std</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>140</v>
+        <v>10033.589</v>
       </c>
       <c r="C4" t="n">
-        <v>59.272</v>
+        <v>6.11</v>
       </c>
       <c r="D4" t="n">
         <v>6.516</v>
       </c>
       <c r="E4" t="n">
-        <v>47.3</v>
+        <v>1.897</v>
       </c>
       <c r="F4" t="n">
-        <v>54.675</v>
+        <v>1002.878</v>
       </c>
       <c r="G4" t="n">
-        <v>58.55</v>
+        <v>6.939</v>
       </c>
       <c r="H4" t="n">
-        <v>64.3</v>
+        <v>7.891</v>
       </c>
       <c r="I4" t="n">
-        <v>82.7</v>
+        <v>7.164</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3.897</v>
+      </c>
+      <c r="K4" t="n">
+        <v>13.496</v>
+      </c>
+      <c r="L4" t="n">
+        <v>21.963</v>
+      </c>
+      <c r="M4" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1.849</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Unemployment_Rate</t>
+          <t>min</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>140</v>
+        <v>6577</v>
       </c>
       <c r="C5" t="n">
-        <v>8.304</v>
+        <v>52.2</v>
       </c>
       <c r="D5" t="n">
-        <v>1.897</v>
+        <v>47.3</v>
       </c>
       <c r="E5" t="n">
         <v>4.5</v>
       </c>
       <c r="F5" t="n">
-        <v>6.9</v>
+        <v>115</v>
       </c>
       <c r="G5" t="n">
-        <v>8.199999999999999</v>
+        <v>17.5</v>
       </c>
       <c r="H5" t="n">
-        <v>9.625</v>
+        <v>4.5</v>
       </c>
       <c r="I5" t="n">
-        <v>14.6</v>
+        <v>5.28</v>
+      </c>
+      <c r="J5" t="n">
+        <v>11.946</v>
+      </c>
+      <c r="K5" t="n">
+        <v>19.59</v>
+      </c>
+      <c r="L5" t="n">
+        <v>11.865</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2.095</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2.425</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Core_Housing_Need</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>140</v>
+        <v>12019.5</v>
       </c>
       <c r="C6" t="n">
-        <v>1720.143</v>
+        <v>59.875</v>
       </c>
       <c r="D6" t="n">
-        <v>1002.878</v>
+        <v>54.675</v>
       </c>
       <c r="E6" t="n">
-        <v>115</v>
+        <v>6.9</v>
       </c>
       <c r="F6" t="n">
         <v>967.5</v>
       </c>
       <c r="G6" t="n">
-        <v>1432.5</v>
+        <v>31.075</v>
       </c>
       <c r="H6" t="n">
-        <v>2287.5</v>
+        <v>14.1</v>
       </c>
       <c r="I6" t="n">
-        <v>5335</v>
+        <v>13.935</v>
+      </c>
+      <c r="J6" t="n">
+        <v>17.425</v>
+      </c>
+      <c r="K6" t="n">
+        <v>31.644</v>
+      </c>
+      <c r="L6" t="n">
+        <v>27.239</v>
+      </c>
+      <c r="M6" t="n">
+        <v>13.557</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.169</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Unaffordable_Housing</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>140</v>
+        <v>16749.5</v>
       </c>
       <c r="C7" t="n">
-        <v>35.072</v>
+        <v>63.6</v>
       </c>
       <c r="D7" t="n">
-        <v>6.939</v>
+        <v>58.55</v>
       </c>
       <c r="E7" t="n">
-        <v>17.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>31.075</v>
+        <v>1432.5</v>
       </c>
       <c r="G7" t="n">
         <v>35.6</v>
       </c>
       <c r="H7" t="n">
-        <v>38.525</v>
+        <v>18.55</v>
       </c>
       <c r="I7" t="n">
-        <v>56.5</v>
+        <v>19.287</v>
+      </c>
+      <c r="J7" t="n">
+        <v>20.979</v>
+      </c>
+      <c r="K7" t="n">
+        <v>45.355</v>
+      </c>
+      <c r="L7" t="n">
+        <v>42.516</v>
+      </c>
+      <c r="M7" t="n">
+        <v>17.655</v>
+      </c>
+      <c r="N7" t="n">
+        <v>5.465</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Low_Income_AfterTax_Pct</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>140</v>
+        <v>23854.5</v>
       </c>
       <c r="C8" t="n">
-        <v>19.514</v>
+        <v>69.125</v>
       </c>
       <c r="D8" t="n">
-        <v>7.891</v>
+        <v>64.3</v>
       </c>
       <c r="E8" t="n">
-        <v>4.5</v>
+        <v>9.625</v>
       </c>
       <c r="F8" t="n">
-        <v>14.1</v>
+        <v>2287.5</v>
       </c>
       <c r="G8" t="n">
-        <v>18.55</v>
+        <v>38.525</v>
       </c>
       <c r="H8" t="n">
         <v>23.95</v>
       </c>
       <c r="I8" t="n">
-        <v>45.5</v>
+        <v>24.384</v>
+      </c>
+      <c r="J8" t="n">
+        <v>23.532</v>
+      </c>
+      <c r="K8" t="n">
+        <v>55.46</v>
+      </c>
+      <c r="L8" t="n">
+        <v>66.08199999999999</v>
+      </c>
+      <c r="M8" t="n">
+        <v>23.749</v>
+      </c>
+      <c r="N8" t="n">
+        <v>6.525</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>max</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>140</v>
+        <v>65913</v>
       </c>
       <c r="C9" t="n">
-        <v>19.209</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>7.164</v>
+        <v>82.7</v>
       </c>
       <c r="E9" t="n">
-        <v>5.28</v>
+        <v>14.6</v>
       </c>
       <c r="F9" t="n">
-        <v>13.935</v>
+        <v>5335</v>
       </c>
       <c r="G9" t="n">
-        <v>19.287</v>
+        <v>56.5</v>
       </c>
       <c r="H9" t="n">
-        <v>24.384</v>
+        <v>45.5</v>
       </c>
       <c r="I9" t="n">
         <v>41.388</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>No_Diploma_Pct</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>140</v>
-      </c>
-      <c r="C10" t="n">
-        <v>20.331</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3.897</v>
-      </c>
-      <c r="E10" t="n">
-        <v>11.946</v>
-      </c>
-      <c r="F10" t="n">
-        <v>17.425</v>
-      </c>
-      <c r="G10" t="n">
-        <v>20.979</v>
-      </c>
-      <c r="H10" t="n">
-        <v>23.532</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="J9" t="n">
         <v>27.707</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Immigrant_Population_Pct</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>140</v>
-      </c>
-      <c r="C11" t="n">
-        <v>44.221</v>
-      </c>
-      <c r="D11" t="n">
-        <v>13.496</v>
-      </c>
-      <c r="E11" t="n">
-        <v>19.59</v>
-      </c>
-      <c r="F11" t="n">
-        <v>31.644</v>
-      </c>
-      <c r="G11" t="n">
-        <v>45.355</v>
-      </c>
-      <c r="H11" t="n">
-        <v>55.46</v>
-      </c>
-      <c r="I11" t="n">
+      <c r="K9" t="n">
         <v>70.828</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Visible_Minority_Pct</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>140</v>
-      </c>
-      <c r="C12" t="n">
-        <v>46.48</v>
-      </c>
-      <c r="D12" t="n">
-        <v>21.963</v>
-      </c>
-      <c r="E12" t="n">
-        <v>11.865</v>
-      </c>
-      <c r="F12" t="n">
-        <v>27.239</v>
-      </c>
-      <c r="G12" t="n">
-        <v>42.516</v>
-      </c>
-      <c r="H12" t="n">
-        <v>66.08199999999999</v>
-      </c>
-      <c r="I12" t="n">
+      <c r="L9" t="n">
         <v>94.705</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Renters_Pct</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>140</v>
-      </c>
-      <c r="C13" t="n">
-        <v>18.972</v>
-      </c>
-      <c r="D13" t="n">
-        <v>8.970000000000001</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2.095</v>
-      </c>
-      <c r="F13" t="n">
-        <v>13.557</v>
-      </c>
-      <c r="G13" t="n">
-        <v>17.655</v>
-      </c>
-      <c r="H13" t="n">
-        <v>23.749</v>
-      </c>
-      <c r="I13" t="n">
+      <c r="M9" t="n">
         <v>46.253</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>Lone_Parent_Families_Pct</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>140</v>
-      </c>
-      <c r="C14" t="n">
-        <v>5.593</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1.849</v>
-      </c>
-      <c r="E14" t="n">
-        <v>2.425</v>
-      </c>
-      <c r="F14" t="n">
-        <v>4.169</v>
-      </c>
-      <c r="G14" t="n">
-        <v>5.465</v>
-      </c>
-      <c r="H14" t="n">
-        <v>6.525</v>
-      </c>
-      <c r="I14" t="n">
+      <c r="N9" t="n">
         <v>11.619</v>
       </c>
     </row>
@@ -957,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1057,11 +1048,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
+          <t>Core_Housing_Need</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.473</v>
+        <v>0.551</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -1075,11 +1066,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Renters_Pct</t>
+          <t>Employment_Rate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.471</v>
+        <v>-0.473</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -1093,11 +1084,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lone_Parent_Families_Pct</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.43</v>
+        <v>0.471</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1111,11 +1102,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
+          <t>Lone_Parent_Families_Pct</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.392</v>
+        <v>0.43</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -1129,11 +1120,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Participation_Rate</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.318</v>
+        <v>-0.392</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1147,16 +1138,34 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Bachelors_Degree_Pct</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.318</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>p &lt; 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>0.169</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>0.045</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>p = 0.045</t>
         </is>
@@ -1173,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1255,11 +1264,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Immigrant_Population_Pct</t>
+          <t>Core_Housing_Need</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.614</v>
+        <v>0.651</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -1273,11 +1282,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
+          <t>Immigrant_Population_Pct</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.518</v>
+        <v>0.614</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -1291,11 +1300,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lone_Parent_Families_Pct</t>
+          <t>Employment_Rate</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.503</v>
+        <v>-0.518</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -1309,11 +1318,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
+          <t>Lone_Parent_Families_Pct</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.452</v>
+        <v>0.503</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1327,11 +1336,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Renters_Pct</t>
+          <t>Participation_Rate</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.403</v>
+        <v>-0.452</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -1345,11 +1354,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.377</v>
+        <v>0.403</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -1363,16 +1372,34 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Bachelors_Degree_Pct</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.377</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>p &lt; 0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>0.29</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>0.001</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>p &lt; 0.001</t>
         </is>
@@ -1389,7 +1416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1400,66 +1427,38 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Pearson_r</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Spearman_rho</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Difference</t>
+          <t>VIF</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Unaffordable_Housing</t>
+          <t>Employment_Rate</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.775</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0.746</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.029</v>
+        <v>3013.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Unemployment_Rate</t>
+          <t>Participation_Rate</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.735</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.758</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-0.023</v>
+        <v>2280.629</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Visible_Minority_Pct</t>
+          <t>Unemployment_Rate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.662</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.717</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-0.055</v>
+        <v>108.01</v>
       </c>
     </row>
     <row r="5">
@@ -1469,45 +1468,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5610000000000001</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.614</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-0.053</v>
+        <v>7.509</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
+          <t>Visible_Minority_Pct</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.473</v>
-      </c>
-      <c r="C6" t="n">
-        <v>-0.518</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.045</v>
+        <v>7.345</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Renters_Pct</t>
+          <t>Bachelors_Degree_Pct</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.471</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.403</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.068</v>
+        <v>5.876</v>
       </c>
     </row>
     <row r="8">
@@ -1517,61 +1498,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.073</v>
+        <v>5.235</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
+          <t>Unaffordable_Housing</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.392</v>
-      </c>
-      <c r="C9" t="n">
-        <v>-0.452</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.06</v>
+        <v>4.429</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bachelors_Degree_Pct</t>
+          <t>Renters_Pct</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.318</v>
-      </c>
-      <c r="C10" t="n">
-        <v>-0.377</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.059</v>
+        <v>4.248</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Core_Housing_Need</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.169</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="D11" t="n">
-        <v>-0.121</v>
+        <v>1.884</v>
       </c>
     </row>
   </sheetData>
@@ -1585,159 +1542,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>VIF</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Interpretation</t>
+          <t>Used in This Study</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Employment_Rate</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2958.368</v>
+          <t>Forward Selection</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Starts with no predictors and adds variables sequentially.</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Very High</t>
+          <t>Considered</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Participation_Rate</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2242.616</v>
+          <t>Backward Elimination</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Starts with all predictors and removes the least significant variables.</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Very High</t>
+          <t>Considered</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Unemployment_Rate</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>105.971</v>
+          <t>Stepwise Regression</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Combines forward selection and backward elimination.</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Very High</t>
+          <t>Considered</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Immigrant_Population_Pct</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>7.265</v>
+          <t>Correlation Analysis</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Identifies variables strongly associated with the response variable.</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Visible_Minority_Pct</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>7.191</v>
+          <t>Variance Inflation Factor (VIF)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Detects multicollinearity among predictor variables.</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Bachelors_Degree_Pct</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>5.866</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Lone_Parent_Families_Pct</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>5.22</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Unaffordable_Housing</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>4.428</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Renters_Pct</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Variables</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Adjusted R²</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>AIC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BIC</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Forward</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="D2" t="n">
+        <v>689.54</v>
+      </c>
+      <c r="E2" t="n">
+        <v>716.015</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2.663</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Backward</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="D3" t="n">
+        <v>679.109</v>
+      </c>
+      <c r="E3" t="n">
+        <v>708.525</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.547</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Stepwise</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="D4" t="n">
+        <v>689.54</v>
+      </c>
+      <c r="E4" t="n">
+        <v>716.015</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.663</v>
       </c>
     </row>
   </sheetData>

</xml_diff>